<commit_message>
Simplificar modelo: fecha automática, solo Tienda+Precio por competidor, una foto por producto
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/plantilla_comparativa.xlsx
+++ b/backend/data/plantilla_comparativa.xlsx
@@ -17,9 +17,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -63,12 +61,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,40 +432,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="12" customWidth="1" min="29" max="29"/>
-    <col width="16" customWidth="1" min="30" max="30"/>
-    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,137 +472,42 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Imagen Producto</t>
+          <t>Tienda 1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Fecha Comparativa</t>
+          <t>Precio Competidor 1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Tienda 1</t>
+          <t>Tienda 2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Producto Competidor 1</t>
+          <t>Precio Competidor 2</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Precio Competidor 1</t>
+          <t>Tienda 3</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Imagen Competidor 1</t>
+          <t>Precio Competidor 3</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Fecha Competidor 1</t>
+          <t>Tienda 4</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Tienda 2</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Producto Competidor 2</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Precio Competidor 2</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Imagen Competidor 2</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Fecha Competidor 2</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Tienda 3</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Producto Competidor 3</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Precio Competidor 3</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Imagen Competidor 3</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Fecha Competidor 3</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Tienda 4</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Producto Competidor 4</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
           <t>Precio Competidor 4</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Imagen Competidor 4</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Fecha Competidor 4</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Tienda 5</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Producto Competidor 5</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Precio Competidor 5</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Imagen Competidor 5</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Fecha Competidor 5</t>
         </is>
       </c>
     </row>
@@ -647,48 +530,32 @@
       <c r="D2" t="n">
         <v>359.9</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>46209</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tottus</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>299.9</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Tottus</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Tequila Patrón Añejo Botella 750 mL</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
+          <t>Plaza Vea</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
         <v>299.9</v>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Plaza Vea</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Tequila PATRON Añejo Botella 700ml</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>299.9</v>
-      </c>
-      <c r="Q2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Wong</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Tequila Patrón Añejo Botella 750 mL</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
+      <c r="J2" t="n">
         <v>349.9</v>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -709,59 +576,36 @@
       <c r="D3" t="n">
         <v>13.9</v>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>46216</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Plaza Vea</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>16.5</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Plaza Vea</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Yogurt Vakimu Natural 1 kg</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
           <t>Tottus</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Yogurt Vakimu Natural 1 kg</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
+      <c r="H3" t="n">
         <v>15.9</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Metro</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Yogurt Vakimu Natural 1 kg</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
+      <c r="J3" t="n">
         <v>16.2</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Wong</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Yogurt Vakimu Natural 1 kg</t>
-        </is>
-      </c>
-      <c r="X3" t="n">
+      <c r="L3" t="n">
         <v>15.5</v>
       </c>
     </row>
@@ -776,18 +620,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Instrucciones rápidas</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -806,68 +653,78 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Marca: marca del producto (se muestra en la tarjeta "Mi producto").</t>
+          <t>3. Producto: nombre del producto, incluyendo su presentación (ej. "Yogurt Vakimu Natural 1 kg").</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. Precio Holi: precio de venta al público vigente en Holi.</t>
+          <t>4. Marca: marca del producto.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5. Imagen Producto / Imagen Competidor N: opcional. Si tienes una URL de foto, pégala aquí y se mostrará automáticamente; si se deja en blanco, se muestra un ícono genérico.</t>
+          <t>5. Precio Holi: precio de venta al público vigente en Holi.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6. Fecha Comparativa: fecha en la que se hizo el Scrapp / comparación de precios (aplica a todo el producto).</t>
+          <t>6. Tienda 1/2/3/4: nombre de la tienda competidora encontrada en el Scrapp (ej. Tottus, Plaza Vea, Metro, Wong).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7. Tienda 1/2/3, Producto Competidor 1/2/3, Precio Competidor 1/2/3: opcional, uno por competidor encontrado. Deja en blanco si no hay dato para ese competidor.</t>
+          <t>7. Precio Competidor 1/2/3/4: precio encontrado en esa tienda. Deja ambas celdas en blanco si no hay dato para ese competidor.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8. Fecha Competidor N: opcional. Si un competidor se revisó en otra fecha distinta a la general, indícala aquí; si se deja en blanco, se usa la Fecha Comparativa general.</t>
+          <t>8. No hace falta escribir el nombre del producto del competidor: se asume que es el mismo que el de Holi.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9. El sistema calcula automáticamente el monto y porcentaje de diferencia ("por encima" o "por debajo") entre el precio Holi y cada competidor. No hay que calcularlo manualmente.</t>
+          <t>9. No hace falta poner fecha: el sistema usa automáticamente la fecha en que subes este archivo.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10. Guarda el archivo con el mismo nombre: plantilla_comparativa.xlsx</t>
+          <t>10. La foto del producto se sube aparte, desde el panel (una sola foto por producto, sección 3).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>11. Entrega el archivo a TI (o colócalo en la carpeta acordada) para que se actualice la web.</t>
+          <t>11. El sistema calcula automáticamente el monto y porcentaje de diferencia ("por encima"/"por debajo") frente a cada competidor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12. Guarda el archivo y súbelo desde el panel /admin, sección "1. Cargar Excel con la comparativa".</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Cualquier duda, contactar al equipo de TI.</t>
         </is>

</xml_diff>

<commit_message>
Facilitar carga de fotos: columna Imagen URL en Excel + carga masiva por ZIP
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/plantilla_comparativa.xlsx
+++ b/backend/data/plantilla_comparativa.xlsx
@@ -432,21 +432,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,40 +473,45 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Imagen URL</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Tienda 1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Precio Competidor 1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tienda 2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Precio Competidor 2</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Tienda 3</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Precio Competidor 3</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Tienda 4</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Precio Competidor 4</t>
         </is>
@@ -530,32 +536,33 @@
       <c r="D2" t="n">
         <v>359.9</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Tottus</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>299.9</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Plaza Vea</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>299.9</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Wong</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>349.9</v>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -576,36 +583,37 @@
       <c r="D3" t="n">
         <v>13.9</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Plaza Vea</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>16.5</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Tottus</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>15.9</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Metro</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>16.2</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Wong</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>15.5</v>
       </c>
     </row>
@@ -620,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -674,57 +682,64 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6. Tienda 1/2/3/4: nombre de la tienda competidora encontrada en el Scrapp (ej. Tottus, Plaza Vea, Metro, Wong).</t>
+          <t>6. Imagen URL: opcional. Si ya tienes un enlace web a la foto del producto (catálogo, Drive público, etc.), pégalo aquí y se usa automáticamente. Si lo dejas en blanco, se conserva la foto que hayas subido antes desde el panel, o se muestra un ícono genérico si no hay ninguna.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7. Precio Competidor 1/2/3/4: precio encontrado en esa tienda. Deja ambas celdas en blanco si no hay dato para ese competidor.</t>
+          <t>7. Tienda 1/2/3/4: nombre de la tienda competidora encontrada en el Scrapp (ej. Tottus, Plaza Vea, Metro, Wong).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8. No hace falta escribir el nombre del producto del competidor: se asume que es el mismo que el de Holi.</t>
+          <t>8. Precio Competidor 1/2/3/4: precio encontrado en esa tienda. Deja ambas celdas en blanco si no hay dato para ese competidor.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9. No hace falta poner fecha: el sistema usa automáticamente la fecha en que subes este archivo.</t>
+          <t>9. No hace falta escribir el nombre del producto del competidor: se asume que es el mismo que el de Holi.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10. La foto del producto se sube aparte, desde el panel (una sola foto por producto, sección 3).</t>
+          <t>10. No hace falta poner fecha: el sistema usa automáticamente la fecha en que subes este archivo.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>11. El sistema calcula automáticamente el monto y porcentaje de diferencia ("por encima"/"por debajo") frente a cada competidor.</t>
+          <t>11. Si no tienes URLs de fotos, también puedes subir un .zip con todas las fotos (nombradas como el SKU) desde la sección 3 del panel, en un solo paso.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12. Guarda el archivo y súbelo desde el panel /admin, sección "1. Cargar Excel con la comparativa".</t>
+          <t>12. El sistema calcula automáticamente el monto y porcentaje de diferencia ("por encima"/"por debajo") frente a cada competidor.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>13. Guarda el archivo y súbelo desde el panel /admin, sección "1. Cargar Excel con la comparativa".</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Cualquier duda, contactar al equipo de TI.</t>
         </is>

</xml_diff>